<commit_message>
update ignore rules dan report assets
</commit_message>
<xml_diff>
--- a/report/hasil_pengujian.xlsx
+++ b/report/hasil_pengujian.xlsx
@@ -2280,16 +2280,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>354.984</v>
+        <v>1488.897</v>
       </c>
       <c r="E2" t="n">
-        <v>341.145</v>
+        <v>1678.413</v>
       </c>
       <c r="F2" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="G2" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="H2" t="n">
         <v>5</v>
@@ -2310,16 +2310,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>330.12</v>
+        <v>801.769</v>
       </c>
       <c r="E3" t="n">
-        <v>334.747</v>
+        <v>800.934</v>
       </c>
       <c r="F3" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="G3" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="H3" t="n">
         <v>5</v>
@@ -2340,16 +2340,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>341.502</v>
+        <v>788.104</v>
       </c>
       <c r="E4" t="n">
-        <v>342.638</v>
+        <v>769.1420000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>2.928</v>
+        <v>1.269</v>
       </c>
       <c r="G4" t="n">
-        <v>2.919</v>
+        <v>1.3</v>
       </c>
       <c r="H4" t="n">
         <v>5</v>
@@ -2370,16 +2370,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>333.422</v>
+        <v>824.66</v>
       </c>
       <c r="E5" t="n">
-        <v>334.812</v>
+        <v>874.837</v>
       </c>
       <c r="F5" t="n">
-        <v>2.999</v>
+        <v>1.213</v>
       </c>
       <c r="G5" t="n">
-        <v>2.987</v>
+        <v>1.143</v>
       </c>
       <c r="H5" t="n">
         <v>5</v>
@@ -2400,16 +2400,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>351.529</v>
+        <v>822.14</v>
       </c>
       <c r="E6" t="n">
-        <v>352.273</v>
+        <v>850.778</v>
       </c>
       <c r="F6" t="n">
-        <v>28.447</v>
+        <v>12.163</v>
       </c>
       <c r="G6" t="n">
-        <v>28.387</v>
+        <v>11.754</v>
       </c>
       <c r="H6" t="n">
         <v>5</v>
@@ -2430,16 +2430,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>365.047</v>
+        <v>985.825</v>
       </c>
       <c r="E7" t="n">
-        <v>373.77</v>
+        <v>894.2910000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>27.394</v>
+        <v>10.144</v>
       </c>
       <c r="G7" t="n">
-        <v>26.754</v>
+        <v>11.182</v>
       </c>
       <c r="H7" t="n">
         <v>5</v>
@@ -2512,10 +2512,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>41.912</v>
+        <v>50.735</v>
       </c>
       <c r="E2" t="n">
-        <v>48.529</v>
+        <v>41.176</v>
       </c>
       <c r="F2" t="n">
         <v>50</v>
@@ -2534,10 +2534,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>50.735</v>
+        <v>52.206</v>
       </c>
       <c r="E3" t="n">
-        <v>48.529</v>
+        <v>44.853</v>
       </c>
       <c r="F3" t="n">
         <v>50</v>
@@ -2556,10 +2556,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>11.706</v>
+        <v>13.889</v>
       </c>
       <c r="E4" t="n">
-        <v>51.19</v>
+        <v>49.603</v>
       </c>
       <c r="F4" t="n">
         <v>50</v>
@@ -2578,10 +2578,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>15.079</v>
+        <v>13.492</v>
       </c>
       <c r="E5" t="n">
-        <v>48.016</v>
+        <v>50.397</v>
       </c>
       <c r="F5" t="n">
         <v>50</v>
@@ -2600,10 +2600,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.803</v>
+        <v>3.217</v>
       </c>
       <c r="E6" t="n">
-        <v>50.597</v>
+        <v>48.3</v>
       </c>
       <c r="F6" t="n">
         <v>50</v>
@@ -2622,10 +2622,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3.079</v>
+        <v>2.757</v>
       </c>
       <c r="E7" t="n">
-        <v>49.586</v>
+        <v>47.932</v>
       </c>
       <c r="F7" t="n">
         <v>50</v>
@@ -2694,7 +2694,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7.989</v>
+        <v>7.9864</v>
       </c>
     </row>
     <row r="4">
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7.988</v>
+        <v>7.9862</v>
       </c>
     </row>
   </sheetData>
@@ -2767,13 +2767,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.928</v>
+        <v>1.269</v>
       </c>
       <c r="C2" t="n">
-        <v>2.919</v>
+        <v>1.3</v>
       </c>
       <c r="D2" t="n">
-        <v>18.807</v>
+        <v>22.614</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2788,13 +2788,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.999</v>
+        <v>1.213</v>
       </c>
       <c r="C3" t="n">
-        <v>2.987</v>
+        <v>1.143</v>
       </c>
       <c r="D3" t="n">
-        <v>22.964</v>
+        <v>22.818</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>

</xml_diff>